<commit_message>
Trailing sweep per-regime top-20 snapshot (run 28009972567)
</commit_message>
<xml_diff>
--- a/sweep_reports/trailing_top20/trailing_top20.xlsx
+++ b/sweep_reports/trailing_top20/trailing_top20.xlsx
@@ -502,26 +502,26 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to1_tc0p1</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>311935.8</v>
+        <v>230146.32</v>
       </c>
       <c r="D2" t="n">
-        <v>79214.91</v>
+        <v>52619.81</v>
       </c>
       <c r="E2" t="n">
-        <v>9.65</v>
+        <v>35.55</v>
       </c>
       <c r="F2" t="n">
-        <v>314297.55</v>
+        <v>232450.47</v>
       </c>
       <c r="G2" t="n">
         <v>1</v>
       </c>
       <c r="H2" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="I2" t="n">
         <v>0.1</v>
@@ -551,26 +551,26 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>to0p1_tc0p2</t>
+          <t>to1_tc0p2</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>304688.85</v>
+        <v>223560.59</v>
       </c>
       <c r="D3" t="n">
-        <v>77037.75999999999</v>
+        <v>50861.66</v>
       </c>
       <c r="E3" t="n">
-        <v>9.720000000000001</v>
+        <v>34.96</v>
       </c>
       <c r="F3" t="n">
-        <v>307050.6</v>
+        <v>225864.74</v>
       </c>
       <c r="G3" t="n">
         <v>1</v>
       </c>
       <c r="H3" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="I3" t="n">
         <v>0.2</v>
@@ -600,26 +600,26 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>to0p2_tc0p1</t>
+          <t>to1_tc0p1</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>303235.97</v>
+        <v>202323.57</v>
       </c>
       <c r="D4" t="n">
-        <v>76469.7</v>
+        <v>45381.99</v>
       </c>
       <c r="E4" t="n">
-        <v>10.39</v>
+        <v>16.19</v>
       </c>
       <c r="F4" t="n">
-        <v>305591.39</v>
+        <v>204479.25</v>
       </c>
       <c r="G4" t="n">
         <v>1</v>
       </c>
       <c r="H4" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I4" t="n">
         <v>0.1</v>
@@ -628,13 +628,13 @@
         <v>8</v>
       </c>
       <c r="K4" t="n">
-        <v>1.15</v>
+        <v>1.9</v>
       </c>
       <c r="L4" t="n">
-        <v>180</v>
+        <v>240</v>
       </c>
       <c r="M4" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="N4" t="n">
         <v>0.25</v>
@@ -649,26 +649,26 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>to0p2_tc0p2</t>
+          <t>to1_tc0p2</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>295981.38</v>
+        <v>195544.62</v>
       </c>
       <c r="D5" t="n">
-        <v>74175.84</v>
+        <v>43542.17</v>
       </c>
       <c r="E5" t="n">
-        <v>13.05</v>
+        <v>16.72</v>
       </c>
       <c r="F5" t="n">
-        <v>298336.8</v>
+        <v>197700.3</v>
       </c>
       <c r="G5" t="n">
         <v>1</v>
       </c>
       <c r="H5" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I5" t="n">
         <v>0.2</v>
@@ -677,13 +677,13 @@
         <v>8</v>
       </c>
       <c r="K5" t="n">
-        <v>1.15</v>
+        <v>1.9</v>
       </c>
       <c r="L5" t="n">
-        <v>180</v>
+        <v>240</v>
       </c>
       <c r="M5" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="N5" t="n">
         <v>0.25</v>
@@ -698,26 +698,26 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to1_tc0p1</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>281732.14</v>
+        <v>168337.44</v>
       </c>
       <c r="D6" t="n">
-        <v>70840.28</v>
+        <v>36018.12</v>
       </c>
       <c r="E6" t="n">
-        <v>8.640000000000001</v>
+        <v>9.779999999999999</v>
       </c>
       <c r="F6" t="n">
-        <v>283960.75</v>
+        <v>170614.74</v>
       </c>
       <c r="G6" t="n">
         <v>1</v>
       </c>
       <c r="H6" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="I6" t="n">
         <v>0.1</v>
@@ -726,16 +726,16 @@
         <v>8</v>
       </c>
       <c r="K6" t="n">
-        <v>1.9</v>
+        <v>2.2</v>
       </c>
       <c r="L6" t="n">
-        <v>240</v>
+        <v>30</v>
       </c>
       <c r="M6" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="N6" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="O6" t="b">
         <v>1</v>
@@ -747,29 +747,29 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>to0p1_tc0p2</t>
+          <t>to1_tc0p1</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>274622.59</v>
+        <v>166904.51</v>
       </c>
       <c r="D7" t="n">
-        <v>68620.42999999999</v>
+        <v>37760.34</v>
       </c>
       <c r="E7" t="n">
-        <v>8.779999999999999</v>
+        <v>31.56</v>
       </c>
       <c r="F7" t="n">
-        <v>276851.2</v>
+        <v>169186.07</v>
       </c>
       <c r="G7" t="n">
         <v>1</v>
       </c>
       <c r="H7" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="I7" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="J7" t="n">
         <v>8</v>
@@ -778,13 +778,13 @@
         <v>1.9</v>
       </c>
       <c r="L7" t="n">
-        <v>240</v>
+        <v>300</v>
       </c>
       <c r="M7" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="O7" t="b">
         <v>1</v>
@@ -796,26 +796,26 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>to0p2_tc0p1</t>
+          <t>to1_tc0p1</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>273049.3</v>
+        <v>164226.39</v>
       </c>
       <c r="D8" t="n">
-        <v>68065.17</v>
+        <v>35836.37</v>
       </c>
       <c r="E8" t="n">
-        <v>9.23</v>
+        <v>6.7</v>
       </c>
       <c r="F8" t="n">
-        <v>275269.36</v>
+        <v>166247.91</v>
       </c>
       <c r="G8" t="n">
         <v>1</v>
       </c>
       <c r="H8" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I8" t="n">
         <v>0.1</v>
@@ -824,16 +824,16 @@
         <v>8</v>
       </c>
       <c r="K8" t="n">
-        <v>1.9</v>
+        <v>2.1</v>
       </c>
       <c r="L8" t="n">
         <v>240</v>
       </c>
       <c r="M8" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="N8" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="O8" t="b">
         <v>1</v>
@@ -845,26 +845,26 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>to0p2_tc0p2</t>
+          <t>to1_tc0p2</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>265671.1</v>
+        <v>162064.25</v>
       </c>
       <c r="D9" t="n">
-        <v>65711.96000000001</v>
+        <v>34375.06</v>
       </c>
       <c r="E9" t="n">
-        <v>9.369999999999999</v>
+        <v>10.3</v>
       </c>
       <c r="F9" t="n">
-        <v>267891.16</v>
+        <v>164341.55</v>
       </c>
       <c r="G9" t="n">
         <v>1</v>
       </c>
       <c r="H9" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I9" t="n">
         <v>0.2</v>
@@ -873,16 +873,16 @@
         <v>8</v>
       </c>
       <c r="K9" t="n">
-        <v>1.9</v>
+        <v>2.2</v>
       </c>
       <c r="L9" t="n">
-        <v>240</v>
+        <v>30</v>
       </c>
       <c r="M9" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="N9" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="O9" t="b">
         <v>1</v>
@@ -894,26 +894,26 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to1_tc0p1</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>238734.43</v>
+        <v>161805.69</v>
       </c>
       <c r="D10" t="n">
-        <v>60555.3</v>
+        <v>35514.72</v>
       </c>
       <c r="E10" t="n">
-        <v>14.06</v>
+        <v>24.55</v>
       </c>
       <c r="F10" t="n">
-        <v>241057.36</v>
+        <v>164062.23</v>
       </c>
       <c r="G10" t="n">
         <v>1</v>
       </c>
       <c r="H10" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="I10" t="n">
         <v>0.1</v>
@@ -925,13 +925,13 @@
         <v>1.9</v>
       </c>
       <c r="L10" t="n">
-        <v>300</v>
+        <v>60</v>
       </c>
       <c r="M10" t="n">
         <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="O10" t="b">
         <v>1</v>
@@ -943,26 +943,26 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to1_tc0p1</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>237956.91</v>
+        <v>161536.52</v>
       </c>
       <c r="D11" t="n">
-        <v>59011.88</v>
+        <v>35295.91</v>
       </c>
       <c r="E11" t="n">
-        <v>2.46</v>
+        <v>28.93</v>
       </c>
       <c r="F11" t="n">
-        <v>240268.23</v>
+        <v>163792.28</v>
       </c>
       <c r="G11" t="n">
         <v>1</v>
       </c>
       <c r="H11" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="I11" t="n">
         <v>0.1</v>
@@ -971,16 +971,16 @@
         <v>8</v>
       </c>
       <c r="K11" t="n">
-        <v>2.2</v>
+        <v>1.15</v>
       </c>
       <c r="L11" t="n">
+        <v>90</v>
+      </c>
+      <c r="M11" t="n">
         <v>30</v>
       </c>
-      <c r="M11" t="n">
-        <v>15</v>
-      </c>
       <c r="N11" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="O11" t="b">
         <v>1</v>
@@ -992,44 +992,44 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to1_tc0p1</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>235337.41</v>
+        <v>159832.66</v>
       </c>
       <c r="D12" t="n">
-        <v>57818.89</v>
+        <v>36622.97</v>
       </c>
       <c r="E12" t="n">
-        <v>20.79</v>
+        <v>10.85</v>
       </c>
       <c r="F12" t="n">
-        <v>237528.82</v>
+        <v>161778.73</v>
       </c>
       <c r="G12" t="n">
         <v>1</v>
       </c>
       <c r="H12" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="I12" t="n">
         <v>0.1</v>
       </c>
       <c r="J12" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K12" t="n">
         <v>1.9</v>
       </c>
       <c r="L12" t="n">
-        <v>240</v>
+        <v>120</v>
       </c>
       <c r="M12" t="n">
         <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="O12" t="b">
         <v>1</v>
@@ -1041,26 +1041,26 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to1_tc0p1</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>232370.43</v>
+        <v>159813.16</v>
       </c>
       <c r="D13" t="n">
-        <v>59536.11</v>
+        <v>35966.37</v>
       </c>
       <c r="E13" t="n">
-        <v>10.95</v>
+        <v>30.93</v>
       </c>
       <c r="F13" t="n">
-        <v>234690.6</v>
+        <v>162095.35</v>
       </c>
       <c r="G13" t="n">
         <v>1</v>
       </c>
       <c r="H13" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="I13" t="n">
         <v>0.1</v>
@@ -1090,26 +1090,26 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to1_tc0p1</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>231740.33</v>
+        <v>159647.54</v>
       </c>
       <c r="D14" t="n">
-        <v>57973.56</v>
+        <v>34831.6</v>
       </c>
       <c r="E14" t="n">
-        <v>7.82</v>
+        <v>5.62</v>
       </c>
       <c r="F14" t="n">
-        <v>234042.65</v>
+        <v>161645</v>
       </c>
       <c r="G14" t="n">
         <v>1</v>
       </c>
       <c r="H14" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="I14" t="n">
         <v>0.1</v>
@@ -1118,16 +1118,16 @@
         <v>8</v>
       </c>
       <c r="K14" t="n">
-        <v>1.15</v>
+        <v>2.3</v>
       </c>
       <c r="L14" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="M14" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="O14" t="b">
         <v>1</v>
@@ -1139,41 +1139,41 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to1_tc0p2</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>231738.68</v>
+        <v>159600.81</v>
       </c>
       <c r="D15" t="n">
-        <v>57191.47</v>
+        <v>36002.06</v>
       </c>
       <c r="E15" t="n">
-        <v>1.35</v>
+        <v>31.82</v>
       </c>
       <c r="F15" t="n">
-        <v>233835.53</v>
+        <v>161882.37</v>
       </c>
       <c r="G15" t="n">
         <v>1</v>
       </c>
       <c r="H15" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="I15" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="J15" t="n">
         <v>8</v>
       </c>
       <c r="K15" t="n">
-        <v>2.1</v>
+        <v>1.9</v>
       </c>
       <c r="L15" t="n">
-        <v>240</v>
+        <v>300</v>
       </c>
       <c r="M15" t="n">
-        <v>24</v>
+        <v>0</v>
       </c>
       <c r="N15" t="n">
         <v>0.5</v>
@@ -1188,44 +1188,44 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to1_tc0p2</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>231542.33</v>
+        <v>157777.18</v>
       </c>
       <c r="D16" t="n">
-        <v>58265.75</v>
+        <v>34039.98</v>
       </c>
       <c r="E16" t="n">
-        <v>11.07</v>
+        <v>7.12</v>
       </c>
       <c r="F16" t="n">
-        <v>233836.43</v>
+        <v>159798.7</v>
       </c>
       <c r="G16" t="n">
         <v>1</v>
       </c>
       <c r="H16" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="I16" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="J16" t="n">
         <v>8</v>
       </c>
       <c r="K16" t="n">
-        <v>1.9</v>
+        <v>2.1</v>
       </c>
       <c r="L16" t="n">
-        <v>60</v>
+        <v>240</v>
       </c>
       <c r="M16" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="N16" t="n">
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="O16" t="b">
         <v>1</v>
@@ -1237,44 +1237,44 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>to0p1_tc0p2</t>
+          <t>to1_tc0p1</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>231423.09</v>
+        <v>157569.39</v>
       </c>
       <c r="D17" t="n">
-        <v>58184.34</v>
+        <v>34260.33</v>
       </c>
       <c r="E17" t="n">
-        <v>14.26</v>
+        <v>18.27</v>
       </c>
       <c r="F17" t="n">
-        <v>233746.02</v>
+        <v>159794.07</v>
       </c>
       <c r="G17" t="n">
         <v>1</v>
       </c>
       <c r="H17" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="I17" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="J17" t="n">
         <v>8</v>
       </c>
       <c r="K17" t="n">
-        <v>1.9</v>
+        <v>1.75</v>
       </c>
       <c r="L17" t="n">
-        <v>300</v>
+        <v>45</v>
       </c>
       <c r="M17" t="n">
         <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="O17" t="b">
         <v>1</v>
@@ -1286,47 +1286,47 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>to0p1_tc2</t>
+          <t>to1_tc0p1</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>231372.06</v>
+        <v>155933.55</v>
       </c>
       <c r="D18" t="n">
-        <v>55582.47</v>
+        <v>34100.28</v>
       </c>
       <c r="E18" t="n">
-        <v>29.59</v>
+        <v>32.03</v>
       </c>
       <c r="F18" t="n">
-        <v>233733.81</v>
+        <v>158097.57</v>
       </c>
       <c r="G18" t="n">
         <v>1</v>
       </c>
       <c r="H18" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="I18" t="n">
-        <v>2</v>
+        <v>0.1</v>
       </c>
       <c r="J18" t="n">
         <v>8</v>
       </c>
       <c r="K18" t="n">
-        <v>1.15</v>
+        <v>2.1</v>
       </c>
       <c r="L18" t="n">
-        <v>180</v>
+        <v>120</v>
       </c>
       <c r="M18" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="N18" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="O18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -1335,26 +1335,26 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>to0p1_tc0p2</t>
+          <t>to1_tc0p2</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>231289.6</v>
+        <v>155545.56</v>
       </c>
       <c r="D19" t="n">
-        <v>56906.01</v>
+        <v>33593.9</v>
       </c>
       <c r="E19" t="n">
-        <v>2.52</v>
+        <v>29.2</v>
       </c>
       <c r="F19" t="n">
-        <v>233600.92</v>
+        <v>157801.32</v>
       </c>
       <c r="G19" t="n">
         <v>1</v>
       </c>
       <c r="H19" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="I19" t="n">
         <v>0.2</v>
@@ -1363,16 +1363,16 @@
         <v>8</v>
       </c>
       <c r="K19" t="n">
-        <v>2.2</v>
+        <v>1.15</v>
       </c>
       <c r="L19" t="n">
+        <v>90</v>
+      </c>
+      <c r="M19" t="n">
         <v>30</v>
       </c>
-      <c r="M19" t="n">
-        <v>15</v>
-      </c>
       <c r="N19" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="O19" t="b">
         <v>1</v>
@@ -1384,29 +1384,29 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>to0p2_tc0p1</t>
+          <t>to1_tc0p2</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>231166.86</v>
+        <v>155310.13</v>
       </c>
       <c r="D20" t="n">
-        <v>58034.81</v>
+        <v>33724.86</v>
       </c>
       <c r="E20" t="n">
-        <v>14.05</v>
+        <v>26.51</v>
       </c>
       <c r="F20" t="n">
-        <v>233485.23</v>
+        <v>157566.67</v>
       </c>
       <c r="G20" t="n">
         <v>1</v>
       </c>
       <c r="H20" t="n">
-        <v>0.2</v>
+        <v>1</v>
       </c>
       <c r="I20" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="J20" t="n">
         <v>8</v>
@@ -1415,13 +1415,13 @@
         <v>1.9</v>
       </c>
       <c r="L20" t="n">
-        <v>300</v>
+        <v>60</v>
       </c>
       <c r="M20" t="n">
         <v>0</v>
       </c>
       <c r="N20" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="O20" t="b">
         <v>1</v>
@@ -1433,26 +1433,26 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to1_tc0p1</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>230683.15</v>
+        <v>154158.38</v>
       </c>
       <c r="D21" t="n">
-        <v>58889.84</v>
+        <v>34933.34</v>
       </c>
       <c r="E21" t="n">
-        <v>7.04</v>
+        <v>29.99</v>
       </c>
       <c r="F21" t="n">
-        <v>232671.13</v>
+        <v>156123.89</v>
       </c>
       <c r="G21" t="n">
         <v>1</v>
       </c>
       <c r="H21" t="n">
-        <v>0.1</v>
+        <v>1</v>
       </c>
       <c r="I21" t="n">
         <v>0.1</v>
@@ -1461,16 +1461,16 @@
         <v>7</v>
       </c>
       <c r="K21" t="n">
-        <v>1.9</v>
+        <v>1.3</v>
       </c>
       <c r="L21" t="n">
-        <v>120</v>
+        <v>90</v>
       </c>
       <c r="M21" t="n">
         <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="O21" t="b">
         <v>1</v>
@@ -1573,20 +1573,20 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p1_tc0p2</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>265670.97</v>
+        <v>252659.84</v>
       </c>
       <c r="D2" t="n">
-        <v>69678.81</v>
+        <v>67251.25</v>
       </c>
       <c r="E2" t="n">
-        <v>37.01</v>
+        <v>38.09</v>
       </c>
       <c r="F2" t="n">
-        <v>270121.06</v>
+        <v>257109.92</v>
       </c>
       <c r="G2" t="n">
         <v>1</v>
@@ -1595,7 +1595,7 @@
         <v>0.1</v>
       </c>
       <c r="I2" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="J2" t="n">
         <v>8</v>
@@ -1626,16 +1626,16 @@
         </is>
       </c>
       <c r="C3" t="n">
-        <v>252659.84</v>
+        <v>226595.55</v>
       </c>
       <c r="D3" t="n">
-        <v>67251.25</v>
+        <v>60689.74</v>
       </c>
       <c r="E3" t="n">
-        <v>38.09</v>
+        <v>18.08</v>
       </c>
       <c r="F3" t="n">
-        <v>257109.92</v>
+        <v>230713.32</v>
       </c>
       <c r="G3" t="n">
         <v>1</v>
@@ -1650,13 +1650,13 @@
         <v>8</v>
       </c>
       <c r="K3" t="n">
-        <v>1.15</v>
+        <v>1.9</v>
       </c>
       <c r="L3" t="n">
-        <v>180</v>
+        <v>240</v>
       </c>
       <c r="M3" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="N3" t="n">
         <v>0.25</v>
@@ -1671,44 +1671,44 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>to0p2_tc0p1</t>
+          <t>to0p1_tc0p2</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>248430.88</v>
+        <v>207468.17</v>
       </c>
       <c r="D4" t="n">
-        <v>66515.07000000001</v>
+        <v>54042.74</v>
       </c>
       <c r="E4" t="n">
-        <v>38.55</v>
+        <v>39.02</v>
       </c>
       <c r="F4" t="n">
-        <v>252851.56</v>
+        <v>211918.25</v>
       </c>
       <c r="G4" t="n">
         <v>1</v>
       </c>
       <c r="H4" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="I4" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="J4" t="n">
         <v>8</v>
       </c>
       <c r="K4" t="n">
-        <v>1.15</v>
+        <v>1.9</v>
       </c>
       <c r="L4" t="n">
-        <v>180</v>
+        <v>300</v>
       </c>
       <c r="M4" t="n">
         <v>0</v>
       </c>
       <c r="N4" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="O4" t="b">
         <v>1</v>
@@ -1720,20 +1720,20 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p1_tc0p2</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>238864.59</v>
+        <v>203998.65</v>
       </c>
       <c r="D5" t="n">
-        <v>62986.82</v>
+        <v>53421.86</v>
       </c>
       <c r="E5" t="n">
-        <v>17.82</v>
+        <v>35.56</v>
       </c>
       <c r="F5" t="n">
-        <v>242982.36</v>
+        <v>208463.19</v>
       </c>
       <c r="G5" t="n">
         <v>1</v>
@@ -1742,25 +1742,25 @@
         <v>0.1</v>
       </c>
       <c r="I5" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="J5" t="n">
         <v>8</v>
       </c>
       <c r="K5" t="n">
-        <v>1.9</v>
+        <v>2.2</v>
       </c>
       <c r="L5" t="n">
         <v>240</v>
       </c>
       <c r="M5" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="N5" t="n">
         <v>0.25</v>
       </c>
       <c r="O5" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -1769,26 +1769,26 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>to0p2_tc0p2</t>
+          <t>to0p1_tc0p2</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>235375.75</v>
+        <v>199466.66</v>
       </c>
       <c r="D6" t="n">
-        <v>63978.64</v>
+        <v>53151.94</v>
       </c>
       <c r="E6" t="n">
-        <v>36.76</v>
+        <v>19.33</v>
       </c>
       <c r="F6" t="n">
-        <v>239796.43</v>
+        <v>203953.01</v>
       </c>
       <c r="G6" t="n">
         <v>1</v>
       </c>
       <c r="H6" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="I6" t="n">
         <v>0.2</v>
@@ -1797,16 +1797,16 @@
         <v>8</v>
       </c>
       <c r="K6" t="n">
-        <v>1.15</v>
+        <v>1.9</v>
       </c>
       <c r="L6" t="n">
-        <v>180</v>
+        <v>60</v>
       </c>
       <c r="M6" t="n">
         <v>0</v>
       </c>
       <c r="N6" t="n">
-        <v>0.25</v>
+        <v>0.75</v>
       </c>
       <c r="O6" t="b">
         <v>1</v>
@@ -1822,16 +1822,16 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>226595.55</v>
+        <v>198986.32</v>
       </c>
       <c r="D7" t="n">
-        <v>60689.74</v>
+        <v>53439.04</v>
       </c>
       <c r="E7" t="n">
-        <v>18.08</v>
+        <v>7.6</v>
       </c>
       <c r="F7" t="n">
-        <v>230713.32</v>
+        <v>203491.27</v>
       </c>
       <c r="G7" t="n">
         <v>1</v>
@@ -1846,16 +1846,16 @@
         <v>8</v>
       </c>
       <c r="K7" t="n">
-        <v>1.9</v>
+        <v>2.2</v>
       </c>
       <c r="L7" t="n">
-        <v>240</v>
+        <v>30</v>
       </c>
       <c r="M7" t="n">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="N7" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="O7" t="b">
         <v>1</v>
@@ -1867,44 +1867,44 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>to0p2_tc0p1</t>
+          <t>to0p1_tc0p2</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>222838.08</v>
+        <v>196625.46</v>
       </c>
       <c r="D8" t="n">
-        <v>59956.01</v>
+        <v>52704.5</v>
       </c>
       <c r="E8" t="n">
-        <v>19.26</v>
+        <v>12.03</v>
       </c>
       <c r="F8" t="n">
-        <v>226920.81</v>
+        <v>200386.35</v>
       </c>
       <c r="G8" t="n">
         <v>1</v>
       </c>
       <c r="H8" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="I8" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="J8" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K8" t="n">
         <v>1.9</v>
       </c>
       <c r="L8" t="n">
-        <v>240</v>
+        <v>120</v>
       </c>
       <c r="M8" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="O8" t="b">
         <v>1</v>
@@ -1916,20 +1916,20 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p1_tc0p2</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>220022.98</v>
+        <v>195271.12</v>
       </c>
       <c r="D9" t="n">
-        <v>56491.64</v>
+        <v>52767.75</v>
       </c>
       <c r="E9" t="n">
-        <v>38.64</v>
+        <v>21.74</v>
       </c>
       <c r="F9" t="n">
-        <v>224473.06</v>
+        <v>199105.81</v>
       </c>
       <c r="G9" t="n">
         <v>1</v>
@@ -1938,22 +1938,22 @@
         <v>0.1</v>
       </c>
       <c r="I9" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="J9" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K9" t="n">
-        <v>1.9</v>
+        <v>1.3</v>
       </c>
       <c r="L9" t="n">
-        <v>300</v>
+        <v>90</v>
       </c>
       <c r="M9" t="n">
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="O9" t="b">
         <v>1</v>
@@ -1965,20 +1965,20 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p1_tc0p2</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>216972.01</v>
+        <v>192735.87</v>
       </c>
       <c r="D10" t="n">
-        <v>55967.98</v>
+        <v>50457.43</v>
       </c>
       <c r="E10" t="n">
-        <v>35.19</v>
+        <v>23.15</v>
       </c>
       <c r="F10" t="n">
-        <v>221436.55</v>
+        <v>197110.08</v>
       </c>
       <c r="G10" t="n">
         <v>1</v>
@@ -1987,25 +1987,25 @@
         <v>0.1</v>
       </c>
       <c r="I10" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="J10" t="n">
         <v>8</v>
       </c>
       <c r="K10" t="n">
-        <v>2.2</v>
+        <v>1.15</v>
       </c>
       <c r="L10" t="n">
-        <v>240</v>
+        <v>90</v>
       </c>
       <c r="M10" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="N10" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="O10" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="11">
@@ -2014,20 +2014,20 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p1_tc0p2</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>211574.43</v>
+        <v>186550.06</v>
       </c>
       <c r="D11" t="n">
-        <v>55438.72</v>
+        <v>49659.86</v>
       </c>
       <c r="E11" t="n">
-        <v>19.08</v>
+        <v>34.87</v>
       </c>
       <c r="F11" t="n">
-        <v>216060.78</v>
+        <v>190591.99</v>
       </c>
       <c r="G11" t="n">
         <v>1</v>
@@ -2036,7 +2036,7 @@
         <v>0.1</v>
       </c>
       <c r="I11" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="J11" t="n">
         <v>8</v>
@@ -2045,13 +2045,13 @@
         <v>1.9</v>
       </c>
       <c r="L11" t="n">
-        <v>60</v>
+        <v>240</v>
       </c>
       <c r="M11" t="n">
         <v>0</v>
       </c>
       <c r="N11" t="n">
-        <v>0.75</v>
+        <v>0.25</v>
       </c>
       <c r="O11" t="b">
         <v>1</v>
@@ -2063,20 +2063,20 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p1_tc0p2</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>210850.07</v>
+        <v>185160.51</v>
       </c>
       <c r="D12" t="n">
-        <v>55864.7</v>
+        <v>49401.45</v>
       </c>
       <c r="E12" t="n">
-        <v>7.54</v>
+        <v>14.26</v>
       </c>
       <c r="F12" t="n">
-        <v>215355.02</v>
+        <v>189438.3</v>
       </c>
       <c r="G12" t="n">
         <v>1</v>
@@ -2085,22 +2085,22 @@
         <v>0.1</v>
       </c>
       <c r="I12" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="J12" t="n">
         <v>8</v>
       </c>
       <c r="K12" t="n">
-        <v>2.2</v>
+        <v>1.75</v>
       </c>
       <c r="L12" t="n">
-        <v>30</v>
+        <v>45</v>
       </c>
       <c r="M12" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="N12" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="O12" t="b">
         <v>1</v>
@@ -2112,26 +2112,26 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>to0p2_tc0p2</t>
+          <t>to0p1_tc0p2</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>210719.07</v>
+        <v>182548.13</v>
       </c>
       <c r="D13" t="n">
-        <v>57696.66</v>
+        <v>50033.06</v>
       </c>
       <c r="E13" t="n">
-        <v>19.6</v>
+        <v>5.21</v>
       </c>
       <c r="F13" t="n">
-        <v>214801.8</v>
+        <v>186304.76</v>
       </c>
       <c r="G13" t="n">
         <v>1</v>
       </c>
       <c r="H13" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="I13" t="n">
         <v>0.2</v>
@@ -2140,16 +2140,16 @@
         <v>8</v>
       </c>
       <c r="K13" t="n">
-        <v>1.9</v>
+        <v>2.1</v>
       </c>
       <c r="L13" t="n">
         <v>240</v>
       </c>
       <c r="M13" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="N13" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="O13" t="b">
         <v>1</v>
@@ -2165,16 +2165,16 @@
         </is>
       </c>
       <c r="C14" t="n">
-        <v>207468.17</v>
+        <v>181258.39</v>
       </c>
       <c r="D14" t="n">
-        <v>54042.74</v>
+        <v>48619.96</v>
       </c>
       <c r="E14" t="n">
-        <v>39.02</v>
+        <v>24.3</v>
       </c>
       <c r="F14" t="n">
-        <v>211918.25</v>
+        <v>185337.07</v>
       </c>
       <c r="G14" t="n">
         <v>1</v>
@@ -2189,19 +2189,19 @@
         <v>8</v>
       </c>
       <c r="K14" t="n">
-        <v>1.9</v>
+        <v>2.1</v>
       </c>
       <c r="L14" t="n">
-        <v>300</v>
+        <v>120</v>
       </c>
       <c r="M14" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="N14" t="n">
         <v>0.5</v>
       </c>
       <c r="O14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -2210,20 +2210,20 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p1_tc0p2</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>206496.26</v>
+        <v>179455.48</v>
       </c>
       <c r="D15" t="n">
-        <v>54553.37</v>
+        <v>47234.38</v>
       </c>
       <c r="E15" t="n">
-        <v>11.86</v>
+        <v>6.28</v>
       </c>
       <c r="F15" t="n">
-        <v>210257.15</v>
+        <v>183346.06</v>
       </c>
       <c r="G15" t="n">
         <v>1</v>
@@ -2232,22 +2232,22 @@
         <v>0.1</v>
       </c>
       <c r="I15" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="J15" t="n">
         <v>7</v>
       </c>
       <c r="K15" t="n">
-        <v>1.9</v>
+        <v>1.45</v>
       </c>
       <c r="L15" t="n">
-        <v>120</v>
+        <v>300</v>
       </c>
       <c r="M15" t="n">
         <v>0</v>
       </c>
       <c r="N15" t="n">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="O15" t="b">
         <v>1</v>
@@ -2259,35 +2259,35 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>to0p2_tc0p1</t>
+          <t>to0p1_tc0p2</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>205669.18</v>
+        <v>178913.15</v>
       </c>
       <c r="D16" t="n">
-        <v>53827.5</v>
+        <v>46489.97</v>
       </c>
       <c r="E16" t="n">
-        <v>39.76</v>
+        <v>12.53</v>
       </c>
       <c r="F16" t="n">
-        <v>210098.14</v>
+        <v>183190.7</v>
       </c>
       <c r="G16" t="n">
         <v>1</v>
       </c>
       <c r="H16" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="I16" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="J16" t="n">
         <v>8</v>
       </c>
       <c r="K16" t="n">
-        <v>1.9</v>
+        <v>2.3</v>
       </c>
       <c r="L16" t="n">
         <v>300</v>
@@ -2296,7 +2296,7 @@
         <v>0</v>
       </c>
       <c r="N16" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="O16" t="b">
         <v>1</v>
@@ -2308,20 +2308,20 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p1_tc0p2</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>205448.59</v>
+        <v>178080.81</v>
       </c>
       <c r="D17" t="n">
-        <v>52981.86</v>
+        <v>49288.88</v>
       </c>
       <c r="E17" t="n">
-        <v>22.23</v>
+        <v>4.65</v>
       </c>
       <c r="F17" t="n">
-        <v>209822.79</v>
+        <v>181743.15</v>
       </c>
       <c r="G17" t="n">
         <v>1</v>
@@ -2330,22 +2330,22 @@
         <v>0.1</v>
       </c>
       <c r="I17" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="J17" t="n">
         <v>8</v>
       </c>
       <c r="K17" t="n">
-        <v>1.15</v>
+        <v>2.3</v>
       </c>
       <c r="L17" t="n">
-        <v>90</v>
+        <v>120</v>
       </c>
       <c r="M17" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="N17" t="n">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="O17" t="b">
         <v>1</v>
@@ -2357,20 +2357,20 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p1_tc0p2</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>204818.03</v>
+        <v>170995.82</v>
       </c>
       <c r="D18" t="n">
-        <v>54482.85</v>
+        <v>45315.37</v>
       </c>
       <c r="E18" t="n">
-        <v>20.92</v>
+        <v>11.64</v>
       </c>
       <c r="F18" t="n">
-        <v>208652.72</v>
+        <v>174551.87</v>
       </c>
       <c r="G18" t="n">
         <v>1</v>
@@ -2379,13 +2379,13 @@
         <v>0.1</v>
       </c>
       <c r="I18" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="J18" t="n">
         <v>7</v>
       </c>
       <c r="K18" t="n">
-        <v>1.3</v>
+        <v>2</v>
       </c>
       <c r="L18" t="n">
         <v>90</v>
@@ -2394,10 +2394,10 @@
         <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="O18" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="19">
@@ -2410,16 +2410,16 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>203998.65</v>
+        <v>170045.9</v>
       </c>
       <c r="D19" t="n">
-        <v>53421.86</v>
+        <v>43979.57</v>
       </c>
       <c r="E19" t="n">
-        <v>35.56</v>
+        <v>34.9</v>
       </c>
       <c r="F19" t="n">
-        <v>208463.19</v>
+        <v>173836.85</v>
       </c>
       <c r="G19" t="n">
         <v>1</v>
@@ -2431,16 +2431,16 @@
         <v>0.2</v>
       </c>
       <c r="J19" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K19" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="L19" t="n">
         <v>240</v>
       </c>
       <c r="M19" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="N19" t="n">
         <v>0.25</v>
@@ -2455,41 +2455,41 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>to0p2_tc0p1</t>
+          <t>to0p1_tc0p2</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>202053.31</v>
+        <v>169102.73</v>
       </c>
       <c r="D20" t="n">
-        <v>53275.06</v>
+        <v>45034.58</v>
       </c>
       <c r="E20" t="n">
-        <v>36.16</v>
+        <v>25.14</v>
       </c>
       <c r="F20" t="n">
-        <v>206496.94</v>
+        <v>172902.26</v>
       </c>
       <c r="G20" t="n">
         <v>1</v>
       </c>
       <c r="H20" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="I20" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="J20" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K20" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="L20" t="n">
-        <v>240</v>
+        <v>60</v>
       </c>
       <c r="M20" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="N20" t="n">
         <v>0.25</v>
@@ -2508,16 +2508,16 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>199466.66</v>
+        <v>166938.05</v>
       </c>
       <c r="D21" t="n">
-        <v>53151.94</v>
+        <v>43513.83</v>
       </c>
       <c r="E21" t="n">
-        <v>19.33</v>
+        <v>25.61</v>
       </c>
       <c r="F21" t="n">
-        <v>203953.01</v>
+        <v>170887.52</v>
       </c>
       <c r="G21" t="n">
         <v>1</v>
@@ -2529,22 +2529,22 @@
         <v>0.2</v>
       </c>
       <c r="J21" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K21" t="n">
-        <v>1.9</v>
+        <v>1.61</v>
       </c>
       <c r="L21" t="n">
-        <v>60</v>
+        <v>180</v>
       </c>
       <c r="M21" t="n">
         <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="O21" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -2644,44 +2644,44 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p2_tc8</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>99647.19</v>
+        <v>58032.02</v>
       </c>
       <c r="D2" t="n">
-        <v>16390.51</v>
+        <v>8589.26</v>
       </c>
       <c r="E2" t="n">
-        <v>31.07</v>
+        <v>32.59</v>
       </c>
       <c r="F2" t="n">
-        <v>103414.83</v>
+        <v>60885.95</v>
       </c>
       <c r="G2" t="n">
-        <v>1</v>
+        <v>0.867</v>
       </c>
       <c r="H2" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I2" t="n">
-        <v>0.1</v>
+        <v>8</v>
       </c>
       <c r="J2" t="n">
         <v>8</v>
       </c>
       <c r="K2" t="n">
-        <v>1.15</v>
+        <v>2.1</v>
       </c>
       <c r="L2" t="n">
-        <v>180</v>
+        <v>240</v>
       </c>
       <c r="M2" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="N2" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="O2" t="b">
         <v>1</v>
@@ -2693,41 +2693,41 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p2_tc8</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>94234.10000000001</v>
+        <v>50639.27</v>
       </c>
       <c r="D3" t="n">
-        <v>14450.64</v>
+        <v>7562.36</v>
       </c>
       <c r="E3" t="n">
-        <v>25.47</v>
+        <v>32.25</v>
       </c>
       <c r="F3" t="n">
-        <v>98090.53999999999</v>
+        <v>53136.29</v>
       </c>
       <c r="G3" t="n">
-        <v>1</v>
+        <v>0.867</v>
       </c>
       <c r="H3" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I3" t="n">
-        <v>0.1</v>
+        <v>8</v>
       </c>
       <c r="J3" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K3" t="n">
-        <v>1.9</v>
+        <v>2.1</v>
       </c>
       <c r="L3" t="n">
-        <v>300</v>
+        <v>240</v>
       </c>
       <c r="M3" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="N3" t="n">
         <v>0.5</v>
@@ -2742,44 +2742,44 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p2_tc8</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>93260.39</v>
+        <v>46929.48</v>
       </c>
       <c r="D4" t="n">
-        <v>15587.7</v>
+        <v>7855.9</v>
       </c>
       <c r="E4" t="n">
-        <v>11.88</v>
+        <v>28.44</v>
       </c>
       <c r="F4" t="n">
-        <v>96588.5</v>
+        <v>49070.01</v>
       </c>
       <c r="G4" t="n">
-        <v>1</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="H4" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I4" t="n">
-        <v>0.1</v>
+        <v>8</v>
       </c>
       <c r="J4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K4" t="n">
-        <v>1.9</v>
+        <v>2.1</v>
       </c>
       <c r="L4" t="n">
-        <v>240</v>
+        <v>300</v>
       </c>
       <c r="M4" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="N4" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="O4" t="b">
         <v>1</v>
@@ -2791,47 +2791,47 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p2_tc8</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>93104.42</v>
+        <v>45142.93</v>
       </c>
       <c r="D5" t="n">
-        <v>14472.95</v>
+        <v>7172.44</v>
       </c>
       <c r="E5" t="n">
-        <v>17.32</v>
+        <v>31.02</v>
       </c>
       <c r="F5" t="n">
-        <v>96990.89</v>
+        <v>47380.24</v>
       </c>
       <c r="G5" t="n">
-        <v>1</v>
+        <v>0.867</v>
       </c>
       <c r="H5" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I5" t="n">
-        <v>0.1</v>
+        <v>8</v>
       </c>
       <c r="J5" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K5" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="L5" t="n">
         <v>240</v>
       </c>
       <c r="M5" t="n">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="N5" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="O5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -2840,44 +2840,44 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>to0p1_tc0p2</t>
+          <t>to0p2_tc8</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>90571.98</v>
+        <v>43841.57</v>
       </c>
       <c r="D6" t="n">
-        <v>14797.28</v>
+        <v>6802.53</v>
       </c>
       <c r="E6" t="n">
-        <v>31.76</v>
+        <v>32.05</v>
       </c>
       <c r="F6" t="n">
-        <v>94339.62</v>
+        <v>46030.64</v>
       </c>
       <c r="G6" t="n">
-        <v>1</v>
+        <v>0.867</v>
       </c>
       <c r="H6" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I6" t="n">
-        <v>0.2</v>
+        <v>8</v>
       </c>
       <c r="J6" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K6" t="n">
-        <v>1.15</v>
+        <v>2.1</v>
       </c>
       <c r="L6" t="n">
-        <v>180</v>
+        <v>240</v>
       </c>
       <c r="M6" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="N6" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="O6" t="b">
         <v>1</v>
@@ -2889,44 +2889,44 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p2_tc8</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>89475.66</v>
+        <v>43443.13</v>
       </c>
       <c r="D7" t="n">
-        <v>13782.41</v>
+        <v>5971.73</v>
       </c>
       <c r="E7" t="n">
-        <v>23.06</v>
+        <v>33.62</v>
       </c>
       <c r="F7" t="n">
-        <v>93427.41</v>
+        <v>45584.26</v>
       </c>
       <c r="G7" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="H7" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I7" t="n">
-        <v>0.1</v>
+        <v>8</v>
       </c>
       <c r="J7" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K7" t="n">
-        <v>1.9</v>
+        <v>2.3</v>
       </c>
       <c r="L7" t="n">
-        <v>60</v>
+        <v>240</v>
       </c>
       <c r="M7" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="N7" t="n">
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="O7" t="b">
         <v>1</v>
@@ -2938,44 +2938,44 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p2_tc8</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>86857.09</v>
+        <v>43309.24</v>
       </c>
       <c r="D8" t="n">
-        <v>13382.89</v>
+        <v>6367.8</v>
       </c>
       <c r="E8" t="n">
-        <v>26.04</v>
+        <v>32.99</v>
       </c>
       <c r="F8" t="n">
-        <v>90147.82000000001</v>
+        <v>45450.37</v>
       </c>
       <c r="G8" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="H8" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I8" t="n">
-        <v>0.1</v>
+        <v>8</v>
       </c>
       <c r="J8" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K8" t="n">
-        <v>1.3</v>
+        <v>2.1</v>
       </c>
       <c r="L8" t="n">
-        <v>90</v>
+        <v>240</v>
       </c>
       <c r="M8" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="N8" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="O8" t="b">
         <v>1</v>
@@ -2987,44 +2987,44 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>to0p2_tc0p1</t>
+          <t>to0p2_tc8</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>86612</v>
+        <v>43092.44</v>
       </c>
       <c r="D9" t="n">
-        <v>14241.5</v>
+        <v>6348.69</v>
       </c>
       <c r="E9" t="n">
-        <v>31.68</v>
+        <v>33.82</v>
       </c>
       <c r="F9" t="n">
-        <v>90333.62</v>
+        <v>45233.57</v>
       </c>
       <c r="G9" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="H9" t="n">
         <v>0.2</v>
       </c>
       <c r="I9" t="n">
-        <v>0.1</v>
+        <v>8</v>
       </c>
       <c r="J9" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K9" t="n">
-        <v>1.15</v>
+        <v>2.2</v>
       </c>
       <c r="L9" t="n">
-        <v>180</v>
+        <v>240</v>
       </c>
       <c r="M9" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="N9" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="O9" t="b">
         <v>1</v>
@@ -3036,44 +3036,44 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p2_tc8</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>85537.41</v>
+        <v>42890.94</v>
       </c>
       <c r="D10" t="n">
-        <v>13254.1</v>
+        <v>6789.35</v>
       </c>
       <c r="E10" t="n">
-        <v>6.85</v>
+        <v>32.95</v>
       </c>
       <c r="F10" t="n">
-        <v>88709.73</v>
+        <v>45032.07</v>
       </c>
       <c r="G10" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="H10" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I10" t="n">
-        <v>0.1</v>
+        <v>8</v>
       </c>
       <c r="J10" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K10" t="n">
-        <v>1.9</v>
+        <v>2</v>
       </c>
       <c r="L10" t="n">
-        <v>120</v>
+        <v>240</v>
       </c>
       <c r="M10" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="N10" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="O10" t="b">
         <v>1</v>
@@ -3085,41 +3085,41 @@
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p2_tc8</t>
         </is>
       </c>
       <c r="C11" t="n">
-        <v>85058.58</v>
+        <v>42801.7</v>
       </c>
       <c r="D11" t="n">
-        <v>13112.25</v>
+        <v>6463.28</v>
       </c>
       <c r="E11" t="n">
-        <v>11.15</v>
+        <v>33.19</v>
       </c>
       <c r="F11" t="n">
-        <v>89015.37</v>
+        <v>44942.83</v>
       </c>
       <c r="G11" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="H11" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I11" t="n">
-        <v>0.1</v>
+        <v>8</v>
       </c>
       <c r="J11" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K11" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="L11" t="n">
-        <v>30</v>
+        <v>240</v>
       </c>
       <c r="M11" t="n">
-        <v>15</v>
+        <v>27</v>
       </c>
       <c r="N11" t="n">
         <v>0.5</v>
@@ -3134,44 +3134,44 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>to0p1_tc0p2</t>
+          <t>to0p2_tc8</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>84641.02</v>
+        <v>42758.6</v>
       </c>
       <c r="D12" t="n">
-        <v>13989.75</v>
+        <v>6405.13</v>
       </c>
       <c r="E12" t="n">
-        <v>13.32</v>
+        <v>33.35</v>
       </c>
       <c r="F12" t="n">
-        <v>87969.13</v>
+        <v>44899.73</v>
       </c>
       <c r="G12" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="H12" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I12" t="n">
-        <v>0.2</v>
+        <v>8</v>
       </c>
       <c r="J12" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K12" t="n">
-        <v>1.9</v>
+        <v>2.1</v>
       </c>
       <c r="L12" t="n">
         <v>240</v>
       </c>
       <c r="M12" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="N12" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="O12" t="b">
         <v>1</v>
@@ -3183,44 +3183,44 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>to0p1_tc0p2</t>
+          <t>to0p2_tc8</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>84552.45</v>
+        <v>42758.6</v>
       </c>
       <c r="D13" t="n">
-        <v>12722.42</v>
+        <v>6405.13</v>
       </c>
       <c r="E13" t="n">
-        <v>28.32</v>
+        <v>33.35</v>
       </c>
       <c r="F13" t="n">
-        <v>88408.89</v>
+        <v>44899.73</v>
       </c>
       <c r="G13" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="H13" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I13" t="n">
-        <v>0.2</v>
+        <v>8</v>
       </c>
       <c r="J13" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K13" t="n">
-        <v>1.9</v>
+        <v>2.1</v>
       </c>
       <c r="L13" t="n">
-        <v>300</v>
+        <v>240</v>
       </c>
       <c r="M13" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="N13" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="O13" t="b">
         <v>1</v>
@@ -3232,47 +3232,47 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>to0p1_tc0p2</t>
+          <t>to0p2_tc8</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>83610.75999999999</v>
+        <v>42758.6</v>
       </c>
       <c r="D14" t="n">
-        <v>12707.17</v>
+        <v>6405.13</v>
       </c>
       <c r="E14" t="n">
-        <v>17.59</v>
+        <v>33.35</v>
       </c>
       <c r="F14" t="n">
-        <v>87497.23</v>
+        <v>44899.73</v>
       </c>
       <c r="G14" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="H14" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I14" t="n">
-        <v>0.2</v>
+        <v>8</v>
       </c>
       <c r="J14" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K14" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="L14" t="n">
         <v>240</v>
       </c>
       <c r="M14" t="n">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="N14" t="n">
         <v>0.25</v>
       </c>
       <c r="O14" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="15">
@@ -3281,41 +3281,41 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>to0p2_tc0p1</t>
+          <t>to0p2_tc8</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>82653.77</v>
+        <v>42585.82</v>
       </c>
       <c r="D15" t="n">
-        <v>12404.22</v>
+        <v>6100.81</v>
       </c>
       <c r="E15" t="n">
-        <v>28.49</v>
+        <v>33.07</v>
       </c>
       <c r="F15" t="n">
-        <v>86477.45</v>
+        <v>44683.27</v>
       </c>
       <c r="G15" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="H15" t="n">
         <v>0.2</v>
       </c>
       <c r="I15" t="n">
-        <v>0.1</v>
+        <v>8</v>
       </c>
       <c r="J15" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K15" t="n">
-        <v>1.9</v>
+        <v>2.1</v>
       </c>
       <c r="L15" t="n">
-        <v>300</v>
+        <v>240</v>
       </c>
       <c r="M15" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="N15" t="n">
         <v>0.5</v>
@@ -3330,44 +3330,44 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p2_tc8</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>82506.92</v>
+        <v>42360.2</v>
       </c>
       <c r="D16" t="n">
-        <v>13018.12</v>
+        <v>6707.72</v>
       </c>
       <c r="E16" t="n">
-        <v>22.11</v>
+        <v>32.62</v>
       </c>
       <c r="F16" t="n">
-        <v>86242.34</v>
+        <v>44501.33</v>
       </c>
       <c r="G16" t="n">
-        <v>1</v>
+        <v>0.867</v>
       </c>
       <c r="H16" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I16" t="n">
-        <v>0.1</v>
+        <v>8</v>
       </c>
       <c r="J16" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K16" t="n">
-        <v>1.15</v>
+        <v>1.9</v>
       </c>
       <c r="L16" t="n">
-        <v>90</v>
+        <v>240</v>
       </c>
       <c r="M16" t="n">
-        <v>30</v>
+        <v>24</v>
       </c>
       <c r="N16" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
       <c r="O16" t="b">
         <v>1</v>
@@ -3379,44 +3379,44 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p2_tc8</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>81890</v>
+        <v>41977.9</v>
       </c>
       <c r="D17" t="n">
-        <v>13486.84</v>
+        <v>6247.34</v>
       </c>
       <c r="E17" t="n">
-        <v>8.82</v>
+        <v>33.38</v>
       </c>
       <c r="F17" t="n">
-        <v>85476.59</v>
+        <v>44119.03</v>
       </c>
       <c r="G17" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="H17" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I17" t="n">
-        <v>0.1</v>
+        <v>8</v>
       </c>
       <c r="J17" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K17" t="n">
-        <v>2.3</v>
+        <v>2.1</v>
       </c>
       <c r="L17" t="n">
-        <v>300</v>
+        <v>240</v>
       </c>
       <c r="M17" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="N17" t="n">
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="O17" t="b">
         <v>1</v>
@@ -3428,47 +3428,47 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>to0p2_tc0p1</t>
+          <t>to0p2_tc8</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>81830.94</v>
+        <v>41188.12</v>
       </c>
       <c r="D18" t="n">
-        <v>12406.83</v>
+        <v>6472.44</v>
       </c>
       <c r="E18" t="n">
-        <v>18.5</v>
+        <v>28.82</v>
       </c>
       <c r="F18" t="n">
-        <v>85684.59</v>
+        <v>43329.52</v>
       </c>
       <c r="G18" t="n">
-        <v>1</v>
+        <v>0.9330000000000001</v>
       </c>
       <c r="H18" t="n">
         <v>0.2</v>
       </c>
       <c r="I18" t="n">
-        <v>0.1</v>
+        <v>8</v>
       </c>
       <c r="J18" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="K18" t="n">
-        <v>2.2</v>
+        <v>2.1</v>
       </c>
       <c r="L18" t="n">
-        <v>240</v>
+        <v>180</v>
       </c>
       <c r="M18" t="n">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="N18" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="O18" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="19">
@@ -3477,44 +3477,44 @@
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p2_tc8</t>
         </is>
       </c>
       <c r="C19" t="n">
-        <v>81447.5</v>
+        <v>39860.19</v>
       </c>
       <c r="D19" t="n">
-        <v>12736.16</v>
+        <v>5817.79</v>
       </c>
       <c r="E19" t="n">
-        <v>5.27</v>
+        <v>33.3</v>
       </c>
       <c r="F19" t="n">
-        <v>84821.39</v>
+        <v>42001.32</v>
       </c>
       <c r="G19" t="n">
-        <v>1</v>
+        <v>0.8</v>
       </c>
       <c r="H19" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I19" t="n">
-        <v>0.1</v>
+        <v>8</v>
       </c>
       <c r="J19" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K19" t="n">
-        <v>1.45</v>
+        <v>2.1</v>
       </c>
       <c r="L19" t="n">
-        <v>300</v>
+        <v>240</v>
       </c>
       <c r="M19" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="N19" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="O19" t="b">
         <v>1</v>
@@ -3526,44 +3526,44 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>to0p2_tc0p1</t>
+          <t>to0p2_tc8</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>81241.82000000001</v>
+        <v>36053.45</v>
       </c>
       <c r="D20" t="n">
-        <v>13258.28</v>
+        <v>5436.14</v>
       </c>
       <c r="E20" t="n">
-        <v>11.18</v>
+        <v>31.37</v>
       </c>
       <c r="F20" t="n">
-        <v>84522.25999999999</v>
+        <v>37839.74</v>
       </c>
       <c r="G20" t="n">
-        <v>1</v>
+        <v>0.867</v>
       </c>
       <c r="H20" t="n">
         <v>0.2</v>
       </c>
       <c r="I20" t="n">
-        <v>0.1</v>
+        <v>8</v>
       </c>
       <c r="J20" t="n">
-        <v>8</v>
+        <v>5</v>
       </c>
       <c r="K20" t="n">
-        <v>1.9</v>
+        <v>2.1</v>
       </c>
       <c r="L20" t="n">
         <v>240</v>
       </c>
       <c r="M20" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="N20" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="O20" t="b">
         <v>1</v>
@@ -3575,47 +3575,47 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p2_tc8</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>80826.00999999999</v>
+        <v>35416.67</v>
       </c>
       <c r="D21" t="n">
-        <v>12550.44</v>
+        <v>7477.81</v>
       </c>
       <c r="E21" t="n">
-        <v>22.48</v>
+        <v>24.35</v>
       </c>
       <c r="F21" t="n">
-        <v>84289.72</v>
+        <v>37558.19</v>
       </c>
       <c r="G21" t="n">
-        <v>1</v>
+        <v>0.867</v>
       </c>
       <c r="H21" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I21" t="n">
-        <v>0.1</v>
+        <v>8</v>
       </c>
       <c r="J21" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="K21" t="n">
-        <v>1.61</v>
+        <v>2.1</v>
       </c>
       <c r="L21" t="n">
-        <v>180</v>
+        <v>120</v>
       </c>
       <c r="M21" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="N21" t="n">
         <v>0.5</v>
       </c>
       <c r="O21" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
   </sheetData>
@@ -3715,26 +3715,26 @@
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p2_tc0p1</t>
         </is>
       </c>
       <c r="C2" t="n">
-        <v>116028.44</v>
+        <v>98348.61</v>
       </c>
       <c r="D2" t="n">
-        <v>3466.6</v>
+        <v>2719.24</v>
       </c>
       <c r="E2" t="n">
-        <v>27.4</v>
+        <v>32.69</v>
       </c>
       <c r="F2" t="n">
-        <v>121019.57</v>
+        <v>103265.19</v>
       </c>
       <c r="G2" t="n">
         <v>1</v>
       </c>
       <c r="H2" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I2" t="n">
         <v>0.1</v>
@@ -3764,26 +3764,26 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p2_tc0p1</t>
         </is>
       </c>
       <c r="C3" t="n">
-        <v>110775.7</v>
+        <v>93904.95</v>
       </c>
       <c r="D3" t="n">
-        <v>3348.87</v>
+        <v>2457.06</v>
       </c>
       <c r="E3" t="n">
-        <v>29.37</v>
+        <v>12.68</v>
       </c>
       <c r="F3" t="n">
-        <v>115895.95</v>
+        <v>98136.36</v>
       </c>
       <c r="G3" t="n">
         <v>1</v>
       </c>
       <c r="H3" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I3" t="n">
         <v>0.1</v>
@@ -3795,13 +3795,13 @@
         <v>1.9</v>
       </c>
       <c r="L3" t="n">
-        <v>300</v>
+        <v>240</v>
       </c>
       <c r="M3" t="n">
-        <v>0</v>
+        <v>20</v>
       </c>
       <c r="N3" t="n">
-        <v>0.5</v>
+        <v>0.25</v>
       </c>
       <c r="O3" t="b">
         <v>1</v>
@@ -3813,26 +3813,26 @@
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p2_tc0p1</t>
         </is>
       </c>
       <c r="C4" t="n">
-        <v>110285.18</v>
+        <v>92004.86</v>
       </c>
       <c r="D4" t="n">
-        <v>3177.51</v>
+        <v>2382.07</v>
       </c>
       <c r="E4" t="n">
-        <v>8.43</v>
+        <v>34.71</v>
       </c>
       <c r="F4" t="n">
-        <v>114596.87</v>
+        <v>97118.24000000001</v>
       </c>
       <c r="G4" t="n">
         <v>1</v>
       </c>
       <c r="H4" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I4" t="n">
         <v>0.1</v>
@@ -3841,19 +3841,19 @@
         <v>8</v>
       </c>
       <c r="K4" t="n">
-        <v>1.9</v>
+        <v>2.2</v>
       </c>
       <c r="L4" t="n">
         <v>240</v>
       </c>
       <c r="M4" t="n">
-        <v>20</v>
+        <v>10</v>
       </c>
       <c r="N4" t="n">
         <v>0.25</v>
       </c>
       <c r="O4" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -3862,26 +3862,26 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p2_tc0p1</t>
         </is>
       </c>
       <c r="C5" t="n">
-        <v>109137.36</v>
+        <v>85665.24000000001</v>
       </c>
       <c r="D5" t="n">
-        <v>3156.07</v>
+        <v>2016.17</v>
       </c>
       <c r="E5" t="n">
-        <v>23.84</v>
+        <v>20.95</v>
       </c>
       <c r="F5" t="n">
-        <v>114307.5</v>
+        <v>90904.17</v>
       </c>
       <c r="G5" t="n">
         <v>1</v>
       </c>
       <c r="H5" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I5" t="n">
         <v>0.1</v>
@@ -3890,19 +3890,19 @@
         <v>8</v>
       </c>
       <c r="K5" t="n">
-        <v>2.2</v>
+        <v>1.9</v>
       </c>
       <c r="L5" t="n">
-        <v>240</v>
+        <v>60</v>
       </c>
       <c r="M5" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="N5" t="n">
-        <v>0.25</v>
+        <v>0.75</v>
       </c>
       <c r="O5" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -3911,38 +3911,38 @@
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>to0p1_tc0p2</t>
+          <t>to0p2_tc0p1</t>
         </is>
       </c>
       <c r="C6" t="n">
-        <v>103027.07</v>
+        <v>84569.27</v>
       </c>
       <c r="D6" t="n">
-        <v>2940.54</v>
+        <v>2318.82</v>
       </c>
       <c r="E6" t="n">
-        <v>35.15</v>
+        <v>20.93</v>
       </c>
       <c r="F6" t="n">
-        <v>108018.2</v>
+        <v>88874.69</v>
       </c>
       <c r="G6" t="n">
         <v>1</v>
       </c>
       <c r="H6" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I6" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="J6" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K6" t="n">
-        <v>1.15</v>
+        <v>1.3</v>
       </c>
       <c r="L6" t="n">
-        <v>180</v>
+        <v>90</v>
       </c>
       <c r="M6" t="n">
         <v>0</v>
@@ -3960,44 +3960,44 @@
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p2_tc0p1</t>
         </is>
       </c>
       <c r="C7" t="n">
-        <v>102986.16</v>
+        <v>84166.86</v>
       </c>
       <c r="D7" t="n">
-        <v>2712.98</v>
+        <v>2300.28</v>
       </c>
       <c r="E7" t="n">
-        <v>16.07</v>
+        <v>7.35</v>
       </c>
       <c r="F7" t="n">
-        <v>108273.24</v>
+        <v>88262.85000000001</v>
       </c>
       <c r="G7" t="n">
         <v>1</v>
       </c>
       <c r="H7" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I7" t="n">
         <v>0.1</v>
       </c>
       <c r="J7" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K7" t="n">
         <v>1.9</v>
       </c>
       <c r="L7" t="n">
-        <v>60</v>
+        <v>120</v>
       </c>
       <c r="M7" t="n">
         <v>0</v>
       </c>
       <c r="N7" t="n">
-        <v>0.75</v>
+        <v>1</v>
       </c>
       <c r="O7" t="b">
         <v>1</v>
@@ -4009,44 +4009,44 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p2_tc0p1</t>
         </is>
       </c>
       <c r="C8" t="n">
-        <v>99767.42999999999</v>
+        <v>81484.85000000001</v>
       </c>
       <c r="D8" t="n">
-        <v>3042.27</v>
+        <v>1862.14</v>
       </c>
       <c r="E8" t="n">
-        <v>16.88</v>
+        <v>14.14</v>
       </c>
       <c r="F8" t="n">
-        <v>104114.97</v>
+        <v>86127.28999999999</v>
       </c>
       <c r="G8" t="n">
         <v>1</v>
       </c>
       <c r="H8" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I8" t="n">
         <v>0.1</v>
       </c>
       <c r="J8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K8" t="n">
-        <v>1.3</v>
+        <v>2.3</v>
       </c>
       <c r="L8" t="n">
-        <v>90</v>
+        <v>300</v>
       </c>
       <c r="M8" t="n">
         <v>0</v>
       </c>
       <c r="N8" t="n">
-        <v>0.25</v>
+        <v>0.75</v>
       </c>
       <c r="O8" t="b">
         <v>1</v>
@@ -4058,26 +4058,26 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p2_tc0p1</t>
         </is>
       </c>
       <c r="C9" t="n">
-        <v>98952.36</v>
+        <v>80898.81</v>
       </c>
       <c r="D9" t="n">
-        <v>2989.49</v>
+        <v>2107.54</v>
       </c>
       <c r="E9" t="n">
-        <v>5.57</v>
+        <v>7.85</v>
       </c>
       <c r="F9" t="n">
-        <v>103098.42</v>
+        <v>85330.44</v>
       </c>
       <c r="G9" t="n">
         <v>1</v>
       </c>
       <c r="H9" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I9" t="n">
         <v>0.1</v>
@@ -4086,16 +4086,16 @@
         <v>7</v>
       </c>
       <c r="K9" t="n">
-        <v>1.9</v>
+        <v>1.45</v>
       </c>
       <c r="L9" t="n">
-        <v>120</v>
+        <v>300</v>
       </c>
       <c r="M9" t="n">
         <v>0</v>
       </c>
       <c r="N9" t="n">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="O9" t="b">
         <v>1</v>
@@ -4107,47 +4107,47 @@
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>to0p1_tc0p2</t>
+          <t>to0p2_tc0p1</t>
         </is>
       </c>
       <c r="C10" t="n">
-        <v>98628.36</v>
+        <v>80216.14</v>
       </c>
       <c r="D10" t="n">
-        <v>2565.65</v>
+        <v>1938.43</v>
       </c>
       <c r="E10" t="n">
-        <v>11.51</v>
+        <v>24.43</v>
       </c>
       <c r="F10" t="n">
-        <v>102940.05</v>
+        <v>84805.78</v>
       </c>
       <c r="G10" t="n">
         <v>1</v>
       </c>
       <c r="H10" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I10" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="J10" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K10" t="n">
-        <v>1.9</v>
+        <v>1.61</v>
       </c>
       <c r="L10" t="n">
-        <v>240</v>
+        <v>180</v>
       </c>
       <c r="M10" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="N10" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="O10" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="11">
@@ -4160,16 +4160,16 @@
         </is>
       </c>
       <c r="C11" t="n">
-        <v>98348.61</v>
+        <v>80196.71000000001</v>
       </c>
       <c r="D11" t="n">
-        <v>2719.24</v>
+        <v>1970.17</v>
       </c>
       <c r="E11" t="n">
-        <v>32.69</v>
+        <v>21.22</v>
       </c>
       <c r="F11" t="n">
-        <v>103265.19</v>
+        <v>85084.16</v>
       </c>
       <c r="G11" t="n">
         <v>1</v>
@@ -4187,13 +4187,13 @@
         <v>1.15</v>
       </c>
       <c r="L11" t="n">
-        <v>180</v>
+        <v>90</v>
       </c>
       <c r="M11" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="N11" t="n">
-        <v>0.25</v>
+        <v>1</v>
       </c>
       <c r="O11" t="b">
         <v>1</v>
@@ -4205,26 +4205,26 @@
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p2_tc0p1</t>
         </is>
       </c>
       <c r="C12" t="n">
-        <v>98100.92</v>
+        <v>80049.37</v>
       </c>
       <c r="D12" t="n">
-        <v>2596.87</v>
+        <v>1600.59</v>
       </c>
       <c r="E12" t="n">
-        <v>9.82</v>
+        <v>8.539999999999999</v>
       </c>
       <c r="F12" t="n">
-        <v>102824.09</v>
+        <v>85293.39999999999</v>
       </c>
       <c r="G12" t="n">
         <v>1</v>
       </c>
       <c r="H12" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I12" t="n">
         <v>0.1</v>
@@ -4233,16 +4233,16 @@
         <v>8</v>
       </c>
       <c r="K12" t="n">
-        <v>2.3</v>
+        <v>2.2</v>
       </c>
       <c r="L12" t="n">
-        <v>300</v>
+        <v>30</v>
       </c>
       <c r="M12" t="n">
-        <v>0</v>
+        <v>15</v>
       </c>
       <c r="N12" t="n">
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="O12" t="b">
         <v>1</v>
@@ -4254,26 +4254,26 @@
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p2_tc0p1</t>
         </is>
       </c>
       <c r="C13" t="n">
-        <v>97653.19</v>
+        <v>77263.82000000001</v>
       </c>
       <c r="D13" t="n">
-        <v>2364.16</v>
+        <v>1913.96</v>
       </c>
       <c r="E13" t="n">
-        <v>6.5</v>
+        <v>37.57</v>
       </c>
       <c r="F13" t="n">
-        <v>102945.04</v>
+        <v>82375.55</v>
       </c>
       <c r="G13" t="n">
         <v>1</v>
       </c>
       <c r="H13" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I13" t="n">
         <v>0.1</v>
@@ -4282,19 +4282,19 @@
         <v>8</v>
       </c>
       <c r="K13" t="n">
-        <v>2.2</v>
+        <v>1.61</v>
       </c>
       <c r="L13" t="n">
-        <v>30</v>
+        <v>120</v>
       </c>
       <c r="M13" t="n">
-        <v>15</v>
+        <v>0</v>
       </c>
       <c r="N13" t="n">
-        <v>0.5</v>
+        <v>0.75</v>
       </c>
       <c r="O13" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="14">
@@ -4303,26 +4303,26 @@
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p2_tc0p1</t>
         </is>
       </c>
       <c r="C14" t="n">
-        <v>96990.02</v>
+        <v>76488.03</v>
       </c>
       <c r="D14" t="n">
-        <v>2725.46</v>
+        <v>1967.07</v>
       </c>
       <c r="E14" t="n">
-        <v>20.94</v>
+        <v>15.39</v>
       </c>
       <c r="F14" t="n">
-        <v>101946.83</v>
+        <v>81310.98</v>
       </c>
       <c r="G14" t="n">
         <v>1</v>
       </c>
       <c r="H14" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I14" t="n">
         <v>0.1</v>
@@ -4334,16 +4334,16 @@
         <v>1.15</v>
       </c>
       <c r="L14" t="n">
-        <v>90</v>
+        <v>300</v>
       </c>
       <c r="M14" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="N14" t="n">
-        <v>1</v>
+        <v>0.25</v>
       </c>
       <c r="O14" t="b">
-        <v>1</v>
+        <v>0</v>
       </c>
     </row>
     <row r="15">
@@ -4352,38 +4352,38 @@
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p2_tc0p1</t>
         </is>
       </c>
       <c r="C15" t="n">
-        <v>95909.98</v>
+        <v>74496.14999999999</v>
       </c>
       <c r="D15" t="n">
-        <v>2881.85</v>
+        <v>1619.35</v>
       </c>
       <c r="E15" t="n">
-        <v>5.12</v>
+        <v>35.27</v>
       </c>
       <c r="F15" t="n">
-        <v>100391.14</v>
+        <v>78627.50999999999</v>
       </c>
       <c r="G15" t="n">
         <v>1</v>
       </c>
       <c r="H15" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I15" t="n">
         <v>0.1</v>
       </c>
       <c r="J15" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K15" t="n">
-        <v>1.45</v>
+        <v>1.9</v>
       </c>
       <c r="L15" t="n">
-        <v>300</v>
+        <v>240</v>
       </c>
       <c r="M15" t="n">
         <v>0</v>
@@ -4401,44 +4401,44 @@
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>to0p1_tc0p2</t>
+          <t>to0p2_tc0p1</t>
         </is>
       </c>
       <c r="C16" t="n">
-        <v>95302.32000000001</v>
+        <v>74256.58</v>
       </c>
       <c r="D16" t="n">
-        <v>2537.37</v>
+        <v>1518.57</v>
       </c>
       <c r="E16" t="n">
-        <v>36.58</v>
+        <v>30.26</v>
       </c>
       <c r="F16" t="n">
-        <v>100472.46</v>
+        <v>79500.19</v>
       </c>
       <c r="G16" t="n">
         <v>1</v>
       </c>
       <c r="H16" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I16" t="n">
-        <v>0.2</v>
+        <v>0.1</v>
       </c>
       <c r="J16" t="n">
         <v>8</v>
       </c>
       <c r="K16" t="n">
-        <v>2.2</v>
+        <v>1.9</v>
       </c>
       <c r="L16" t="n">
-        <v>240</v>
+        <v>45</v>
       </c>
       <c r="M16" t="n">
-        <v>10</v>
+        <v>30</v>
       </c>
       <c r="N16" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="O16" t="b">
         <v>0</v>
@@ -4450,47 +4450,47 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p2_tc0p1</t>
         </is>
       </c>
       <c r="C17" t="n">
-        <v>95103.46000000001</v>
+        <v>73512.46000000001</v>
       </c>
       <c r="D17" t="n">
-        <v>2609.08</v>
+        <v>1626.55</v>
       </c>
       <c r="E17" t="n">
-        <v>18.26</v>
+        <v>4.01</v>
       </c>
       <c r="F17" t="n">
-        <v>99734.32000000001</v>
+        <v>77039.28999999999</v>
       </c>
       <c r="G17" t="n">
         <v>1</v>
       </c>
       <c r="H17" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I17" t="n">
         <v>0.1</v>
       </c>
       <c r="J17" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="K17" t="n">
-        <v>1.61</v>
+        <v>2.1</v>
       </c>
       <c r="L17" t="n">
-        <v>180</v>
+        <v>240</v>
       </c>
       <c r="M17" t="n">
-        <v>0</v>
+        <v>24</v>
       </c>
       <c r="N17" t="n">
         <v>0.5</v>
       </c>
       <c r="O17" t="b">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="18">
@@ -4499,44 +4499,44 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p2_tc0p1</t>
         </is>
       </c>
       <c r="C18" t="n">
-        <v>95060.3</v>
+        <v>72790.05</v>
       </c>
       <c r="D18" t="n">
-        <v>2631.21</v>
+        <v>1633.09</v>
       </c>
       <c r="E18" t="n">
-        <v>31.98</v>
+        <v>9.210000000000001</v>
       </c>
       <c r="F18" t="n">
-        <v>100228.13</v>
+        <v>76794.50999999999</v>
       </c>
       <c r="G18" t="n">
         <v>1</v>
       </c>
       <c r="H18" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I18" t="n">
         <v>0.1</v>
       </c>
       <c r="J18" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K18" t="n">
-        <v>1.61</v>
+        <v>1.45</v>
       </c>
       <c r="L18" t="n">
-        <v>120</v>
+        <v>240</v>
       </c>
       <c r="M18" t="n">
         <v>0</v>
       </c>
       <c r="N18" t="n">
-        <v>0.75</v>
+        <v>0.5</v>
       </c>
       <c r="O18" t="b">
         <v>0</v>
@@ -4552,16 +4552,16 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>93904.95</v>
+        <v>72542.34</v>
       </c>
       <c r="D19" t="n">
-        <v>2457.06</v>
+        <v>1553.65</v>
       </c>
       <c r="E19" t="n">
-        <v>12.68</v>
+        <v>17.3</v>
       </c>
       <c r="F19" t="n">
-        <v>98136.36</v>
+        <v>77185.02</v>
       </c>
       <c r="G19" t="n">
         <v>1</v>
@@ -4576,16 +4576,16 @@
         <v>8</v>
       </c>
       <c r="K19" t="n">
-        <v>1.9</v>
+        <v>1.75</v>
       </c>
       <c r="L19" t="n">
-        <v>240</v>
+        <v>45</v>
       </c>
       <c r="M19" t="n">
-        <v>20</v>
+        <v>0</v>
       </c>
       <c r="N19" t="n">
-        <v>0.25</v>
+        <v>0.75</v>
       </c>
       <c r="O19" t="b">
         <v>1</v>
@@ -4597,26 +4597,26 @@
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p2_tc0p1</t>
         </is>
       </c>
       <c r="C20" t="n">
-        <v>93605.71000000001</v>
+        <v>71887.94</v>
       </c>
       <c r="D20" t="n">
-        <v>2751.22</v>
+        <v>1553.72</v>
       </c>
       <c r="E20" t="n">
-        <v>9.76</v>
+        <v>31.45</v>
       </c>
       <c r="F20" t="n">
-        <v>98495.56</v>
+        <v>76015.73</v>
       </c>
       <c r="G20" t="n">
         <v>1</v>
       </c>
       <c r="H20" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I20" t="n">
         <v>0.1</v>
@@ -4625,16 +4625,16 @@
         <v>8</v>
       </c>
       <c r="K20" t="n">
-        <v>1.15</v>
+        <v>2.1</v>
       </c>
       <c r="L20" t="n">
-        <v>300</v>
+        <v>120</v>
       </c>
       <c r="M20" t="n">
-        <v>0</v>
+        <v>30</v>
       </c>
       <c r="N20" t="n">
-        <v>0.25</v>
+        <v>0.5</v>
       </c>
       <c r="O20" t="b">
         <v>0</v>
@@ -4646,44 +4646,44 @@
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>to0p1_tc0p1</t>
+          <t>to0p2_tc0p1</t>
         </is>
       </c>
       <c r="C21" t="n">
-        <v>92364.16</v>
+        <v>71040.22</v>
       </c>
       <c r="D21" t="n">
-        <v>2273.29</v>
+        <v>1889.25</v>
       </c>
       <c r="E21" t="n">
-        <v>20.75</v>
+        <v>13.3</v>
       </c>
       <c r="F21" t="n">
-        <v>97655.77</v>
+        <v>74732.2</v>
       </c>
       <c r="G21" t="n">
         <v>1</v>
       </c>
       <c r="H21" t="n">
-        <v>0.1</v>
+        <v>0.2</v>
       </c>
       <c r="I21" t="n">
         <v>0.1</v>
       </c>
       <c r="J21" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="K21" t="n">
-        <v>1.9</v>
+        <v>2</v>
       </c>
       <c r="L21" t="n">
-        <v>45</v>
+        <v>90</v>
       </c>
       <c r="M21" t="n">
-        <v>30</v>
+        <v>0</v>
       </c>
       <c r="N21" t="n">
-        <v>0.5</v>
+        <v>1</v>
       </c>
       <c r="O21" t="b">
         <v>0</v>

</xml_diff>